<commit_message>
Registrato bug in testbook
</commit_message>
<xml_diff>
--- a/docs/testbook/ClinicaFlow_TestBook_API.xlsx
+++ b/docs/testbook/ClinicaFlow_TestBook_API.xlsx
@@ -8,20 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\valen\clinicaflow\docs\testbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B829CA6-33F3-4444-B0F3-1115C5D9F990}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28B8CB74-FAEE-4705-BC84-56E602C9B112}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20370" yWindow="-4770" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{1C9960E8-B103-4EFA-9509-2FD0D5F86CF0}"/>
   </bookViews>
   <sheets>
     <sheet name="ClinicaFlow_TestBook_API" sheetId="1" r:id="rId1"/>
-    <sheet name="TS1_20260321" sheetId="2" r:id="rId2"/>
+    <sheet name="BUG" sheetId="3" r:id="rId2"/>
+    <sheet name="TS1_20260321" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="166">
   <si>
     <t>ID Test</t>
   </si>
@@ -498,6 +499,27 @@
   </si>
   <si>
     <t>Non è possibile eliminare una specializzazione associata a uno o più medici.</t>
+  </si>
+  <si>
+    <t>ID Bug</t>
+  </si>
+  <si>
+    <t>Errore</t>
+  </si>
+  <si>
+    <t>Priorità</t>
+  </si>
+  <si>
+    <t>ALTA</t>
+  </si>
+  <si>
+    <t>TS1_20260321</t>
+  </si>
+  <si>
+    <t>Sessione OK</t>
+  </si>
+  <si>
+    <t>Sessione KO</t>
   </si>
 </sst>
 </file>
@@ -640,7 +662,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -820,8 +842,20 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor theme="4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor theme="4" tint="0.59999389629810485"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -936,6 +970,69 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top/>
+      <bottom style="thick">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top/>
+      <bottom style="thick">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -981,7 +1078,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -991,6 +1088,33 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="33" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1037,91 +1161,7 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="48">
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
+  <dxfs count="38">
     <dxf>
       <fill>
         <patternFill>
@@ -1146,7 +1186,14 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FF92D050"/>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1167,21 +1214,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
+          <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1200,67 +1233,88 @@
       </fill>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1276,42 +1330,42 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5E234CF2-B3FB-42E4-9C2F-2101E3219E96}" name="Table1" displayName="Table1" ref="A1:L24" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5E234CF2-B3FB-42E4-9C2F-2101E3219E96}" name="Table1" displayName="Table1" ref="A1:L24" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36">
   <autoFilter ref="A1:L24" xr:uid="{5E234CF2-B3FB-42E4-9C2F-2101E3219E96}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{3860FCCE-8AB2-4BA5-A927-55A78AF301A2}" name="ID Test" dataDxfId="27"/>
-    <tableColumn id="2" xr3:uid="{6B8298D4-C558-435B-BC50-DF9FF417402B}" name="Area" dataDxfId="26"/>
-    <tableColumn id="3" xr3:uid="{53DE22B4-8437-4EA6-813E-2F0CF7E72133}" name="Obiettivo" dataDxfId="25"/>
-    <tableColumn id="4" xr3:uid="{59024008-94B6-47E6-8C7F-69725DFAE6EC}" name="Endpoint" dataDxfId="24"/>
-    <tableColumn id="5" xr3:uid="{DC8ACE73-D608-4E52-81FB-F85282B31F51}" name="Metodo HTTP" dataDxfId="23"/>
-    <tableColumn id="6" xr3:uid="{E583E0AB-6285-4FCA-BC35-0CD0BFB6F457}" name="Payload JSON" dataDxfId="22"/>
-    <tableColumn id="7" xr3:uid="{5BDBA1B2-61ED-47D6-88D1-CDE3D8CC9212}" name="Risultato atteso - Status Code" dataDxfId="21"/>
-    <tableColumn id="8" xr3:uid="{F14E32B9-432F-43ED-9E31-411BF4ADBC3F}" name="Risultato atteso - Dettaglio" dataDxfId="20"/>
-    <tableColumn id="9" xr3:uid="{DFDF46B3-7AFF-4643-9EAB-E56F926CE154}" name="Esito" dataDxfId="19"/>
-    <tableColumn id="10" xr3:uid="{5192CEE0-B98B-4E21-8BEA-8F62C2DAC458}" name="Risultato ottenuto" dataDxfId="18"/>
-    <tableColumn id="11" xr3:uid="{E9C64C9D-7B98-4D7D-8A82-64CB9D831A1C}" name="Screenshot" dataDxfId="17"/>
-    <tableColumn id="12" xr3:uid="{D98AF63F-322C-4828-B53E-197F74FEE6FE}" name="Note" dataDxfId="16"/>
+    <tableColumn id="1" xr3:uid="{3860FCCE-8AB2-4BA5-A927-55A78AF301A2}" name="ID Test" dataDxfId="35"/>
+    <tableColumn id="2" xr3:uid="{6B8298D4-C558-435B-BC50-DF9FF417402B}" name="Area" dataDxfId="34"/>
+    <tableColumn id="3" xr3:uid="{53DE22B4-8437-4EA6-813E-2F0CF7E72133}" name="Obiettivo" dataDxfId="33"/>
+    <tableColumn id="4" xr3:uid="{59024008-94B6-47E6-8C7F-69725DFAE6EC}" name="Endpoint" dataDxfId="32"/>
+    <tableColumn id="5" xr3:uid="{DC8ACE73-D608-4E52-81FB-F85282B31F51}" name="Metodo HTTP" dataDxfId="31"/>
+    <tableColumn id="6" xr3:uid="{E583E0AB-6285-4FCA-BC35-0CD0BFB6F457}" name="Payload JSON" dataDxfId="30"/>
+    <tableColumn id="7" xr3:uid="{5BDBA1B2-61ED-47D6-88D1-CDE3D8CC9212}" name="Risultato atteso - Status Code" dataDxfId="29"/>
+    <tableColumn id="8" xr3:uid="{F14E32B9-432F-43ED-9E31-411BF4ADBC3F}" name="Risultato atteso - Dettaglio" dataDxfId="28"/>
+    <tableColumn id="9" xr3:uid="{DFDF46B3-7AFF-4643-9EAB-E56F926CE154}" name="Esito" dataDxfId="27"/>
+    <tableColumn id="10" xr3:uid="{5192CEE0-B98B-4E21-8BEA-8F62C2DAC458}" name="Risultato ottenuto" dataDxfId="26"/>
+    <tableColumn id="11" xr3:uid="{E9C64C9D-7B98-4D7D-8A82-64CB9D831A1C}" name="Screenshot" dataDxfId="25"/>
+    <tableColumn id="12" xr3:uid="{D98AF63F-322C-4828-B53E-197F74FEE6FE}" name="Note" dataDxfId="24"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5EC5406F-ABEC-4C5A-BB6C-648C616B89A5}" name="Table13" displayName="Table13" ref="A1:L24" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5EC5406F-ABEC-4C5A-BB6C-648C616B89A5}" name="Table13" displayName="Table13" ref="A1:L24" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
   <autoFilter ref="A1:L24" xr:uid="{5E234CF2-B3FB-42E4-9C2F-2101E3219E96}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{5009D189-63E8-4852-A288-87D6EC1E7033}" name="ID Test" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{84642470-32B1-46DB-88F2-1BC4AE8F75C8}" name="Area" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{4F14914F-A3C4-4267-A392-EC2D02D6ADDF}" name="Obiettivo" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{62A87606-C1B8-47E6-9530-D288374DCDF3}" name="Endpoint" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{19E09EE6-EB67-45CF-9A03-E0F0523DB6A0}" name="Metodo HTTP" dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{A7AC84FA-A2F1-4930-BDDD-E380EE204368}" name="Payload JSON" dataDxfId="8"/>
-    <tableColumn id="7" xr3:uid="{25C18B10-E594-4E87-AD84-2A557086D8F7}" name="Risultato atteso - Status Code" dataDxfId="7"/>
-    <tableColumn id="8" xr3:uid="{94B79096-6200-43FE-8F50-1C48EB575740}" name="Risultato atteso - Dettaglio" dataDxfId="6"/>
-    <tableColumn id="9" xr3:uid="{AD4E1447-793D-4E65-9313-6A19D961F6AE}" name="Esito" dataDxfId="5"/>
-    <tableColumn id="10" xr3:uid="{B18252F9-BB1D-47B7-8E2C-F42387EC3664}" name="Risultato ottenuto" dataDxfId="4"/>
-    <tableColumn id="11" xr3:uid="{15A8AB07-0563-4A1C-839B-92039F98E2D5}" name="Screenshot" dataDxfId="3"/>
-    <tableColumn id="12" xr3:uid="{4BA21C77-65A7-407A-A5E1-0AA6154386E8}" name="Note" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{5009D189-63E8-4852-A288-87D6EC1E7033}" name="ID Test" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{84642470-32B1-46DB-88F2-1BC4AE8F75C8}" name="Area" dataDxfId="20"/>
+    <tableColumn id="3" xr3:uid="{4F14914F-A3C4-4267-A392-EC2D02D6ADDF}" name="Obiettivo" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{62A87606-C1B8-47E6-9530-D288374DCDF3}" name="Endpoint" dataDxfId="18"/>
+    <tableColumn id="5" xr3:uid="{19E09EE6-EB67-45CF-9A03-E0F0523DB6A0}" name="Metodo HTTP" dataDxfId="17"/>
+    <tableColumn id="6" xr3:uid="{A7AC84FA-A2F1-4930-BDDD-E380EE204368}" name="Payload JSON" dataDxfId="16"/>
+    <tableColumn id="7" xr3:uid="{25C18B10-E594-4E87-AD84-2A557086D8F7}" name="Risultato atteso - Status Code" dataDxfId="15"/>
+    <tableColumn id="8" xr3:uid="{94B79096-6200-43FE-8F50-1C48EB575740}" name="Risultato atteso - Dettaglio" dataDxfId="12"/>
+    <tableColumn id="9" xr3:uid="{AD4E1447-793D-4E65-9313-6A19D961F6AE}" name="Esito" dataDxfId="10"/>
+    <tableColumn id="10" xr3:uid="{B18252F9-BB1D-47B7-8E2C-F42387EC3664}" name="Risultato ottenuto" dataDxfId="11"/>
+    <tableColumn id="11" xr3:uid="{15A8AB07-0563-4A1C-839B-92039F98E2D5}" name="Screenshot" dataDxfId="14"/>
+    <tableColumn id="12" xr3:uid="{4BA21C77-65A7-407A-A5E1-0AA6154386E8}" name="Note" dataDxfId="13"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2299,43 +2353,11 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:I10">
-    <cfRule type="cellIs" dxfId="47" priority="10" operator="equal">
-      <formula>"KO"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="46" priority="9" operator="equal">
+  <conditionalFormatting sqref="I2:I24">
+    <cfRule type="cellIs" dxfId="6" priority="1" operator="equal">
       <formula>"OK"</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I11:I19">
-    <cfRule type="cellIs" dxfId="44" priority="7" operator="equal">
-      <formula>"OK"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="45" priority="8" operator="equal">
-      <formula>"KO"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I20">
-    <cfRule type="cellIs" dxfId="42" priority="5" operator="equal">
-      <formula>"OK"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="43" priority="6" operator="equal">
-      <formula>"KO"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I21">
-    <cfRule type="cellIs" dxfId="40" priority="3" operator="equal">
-      <formula>"OK"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="41" priority="4" operator="equal">
-      <formula>"KO"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I22:I24">
-    <cfRule type="cellIs" dxfId="39" priority="1" operator="equal">
-      <formula>"OK"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="38" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="2" operator="equal">
       <formula>"KO"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2353,6 +2375,107 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27CCBE7D-F26A-41C6-96A8-43D2BF97BCE3}">
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr defaultColWidth="91.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.28515625" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="68.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="89.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="I1" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="11" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="30.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>162</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="H2" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="J2" s="9" t="s">
+        <v>135</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="D2">
+    <cfRule type="cellIs" dxfId="4" priority="1" operator="equal">
+      <formula>"BASSA"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="2" operator="equal">
+      <formula>"MEDIA"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
+      <formula>"ALTA"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2" xr:uid="{78C482C4-A569-4755-A44B-F5FA399B9D9D}">
+      <formula1>"ALTA,MEDIA,BASSA"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FD9EF9F-CB0B-4D0D-A402-0DE892E54EC1}">
   <dimension ref="A1:L24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2365,7 +2488,7 @@
     <col min="6" max="6" width="54.7109375" style="1" customWidth="1"/>
     <col min="7" max="7" width="29" style="2" customWidth="1"/>
     <col min="8" max="8" width="41.7109375" style="1" customWidth="1"/>
-    <col min="9" max="9" width="7.42578125" style="3" customWidth="1"/>
+    <col min="9" max="9" width="7.42578125" style="4" customWidth="1"/>
     <col min="10" max="10" width="41.7109375" style="1" customWidth="1"/>
     <col min="11" max="11" width="58.28515625" style="2" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="64" style="1" bestFit="1" customWidth="1"/>
@@ -2397,7 +2520,7 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="4" t="s">
         <v>8</v>
       </c>
       <c r="J1" s="1" t="s">
@@ -2435,7 +2558,7 @@
       <c r="H2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="4" t="s">
         <v>123</v>
       </c>
       <c r="J2" s="1" t="s">
@@ -2470,7 +2593,7 @@
       <c r="H3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="I3" s="4" t="s">
         <v>123</v>
       </c>
       <c r="J3" s="1" t="s">
@@ -2502,7 +2625,7 @@
       <c r="H4" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="4" t="s">
         <v>123</v>
       </c>
       <c r="J4" s="1" t="s">
@@ -2534,7 +2657,7 @@
       <c r="H5" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="I5" s="4" t="s">
         <v>123</v>
       </c>
       <c r="J5" s="1" t="s">
@@ -2566,7 +2689,7 @@
       <c r="H6" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="I6" s="3" t="s">
+      <c r="I6" s="4" t="s">
         <v>123</v>
       </c>
       <c r="J6" s="1" t="s">
@@ -2604,7 +2727,7 @@
       <c r="H7" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="I7" s="3" t="s">
+      <c r="I7" s="4" t="s">
         <v>123</v>
       </c>
       <c r="J7" s="1" t="s">
@@ -2639,7 +2762,7 @@
       <c r="H8" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="I8" s="3" t="s">
+      <c r="I8" s="4" t="s">
         <v>134</v>
       </c>
       <c r="J8" s="1" t="s">
@@ -2677,7 +2800,7 @@
       <c r="H9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="I9" s="3" t="s">
+      <c r="I9" s="4" t="s">
         <v>123</v>
       </c>
       <c r="J9" s="1" t="s">
@@ -2715,7 +2838,7 @@
       <c r="H10" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="I10" s="3" t="s">
+      <c r="I10" s="4" t="s">
         <v>123</v>
       </c>
       <c r="J10" s="1" t="s">
@@ -2840,7 +2963,7 @@
       <c r="H14" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="I14" s="3" t="s">
+      <c r="I14" s="4" t="s">
         <v>123</v>
       </c>
       <c r="J14" s="1" t="s">
@@ -3008,7 +3131,7 @@
       <c r="H20" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="I20" s="3" t="s">
+      <c r="I20" s="4" t="s">
         <v>123</v>
       </c>
       <c r="J20" s="1" t="s">
@@ -3043,7 +3166,7 @@
       <c r="H21" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="I21" s="3" t="s">
+      <c r="I21" s="4" t="s">
         <v>123</v>
       </c>
       <c r="J21" s="1" t="s">
@@ -3138,43 +3261,11 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:I10">
-    <cfRule type="cellIs" dxfId="36" priority="9" operator="equal">
+  <conditionalFormatting sqref="I2:I24">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"OK"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="10" operator="equal">
-      <formula>"KO"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I11:I19">
-    <cfRule type="cellIs" dxfId="35" priority="7" operator="equal">
-      <formula>"OK"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="34" priority="8" operator="equal">
-      <formula>"KO"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I20">
-    <cfRule type="cellIs" dxfId="33" priority="5" operator="equal">
-      <formula>"OK"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="32" priority="6" operator="equal">
-      <formula>"KO"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I21">
-    <cfRule type="cellIs" dxfId="31" priority="3" operator="equal">
-      <formula>"OK"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="4" operator="equal">
-      <formula>"KO"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I22:I24">
-    <cfRule type="cellIs" dxfId="29" priority="1" operator="equal">
-      <formula>"OK"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
       <formula>"KO"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Bugfixing BUG01 e BUG02
</commit_message>
<xml_diff>
--- a/docs/testbook/ClinicaFlow_TestBook_API.xlsx
+++ b/docs/testbook/ClinicaFlow_TestBook_API.xlsx
@@ -8,21 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\valen\clinicaflow\docs\testbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28B8CB74-FAEE-4705-BC84-56E602C9B112}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99819984-289C-4DA6-AE98-9D390E4B0077}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-4770" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{1C9960E8-B103-4EFA-9509-2FD0D5F86CF0}"/>
+    <workbookView xWindow="20370" yWindow="-4770" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{1C9960E8-B103-4EFA-9509-2FD0D5F86CF0}"/>
   </bookViews>
   <sheets>
     <sheet name="ClinicaFlow_TestBook_API" sheetId="1" r:id="rId1"/>
     <sheet name="BUG" sheetId="3" r:id="rId2"/>
     <sheet name="TS1_20260321" sheetId="2" r:id="rId3"/>
+    <sheet name="TS2_20260321" sheetId="4" r:id="rId4"/>
+    <sheet name="TS3_20260321" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="950" uniqueCount="174">
   <si>
     <t>ID Test</t>
   </si>
@@ -520,6 +522,44 @@
   </si>
   <si>
     <t>Sessione KO</t>
+  </si>
+  <si>
+    <t>{
+  "firstName": "Mario",
+  "lastName": "Rossi",
+  "taxCode": "RSSMRA85D12H501X",
+  "dateOfBirth": "1985-04-12T00:00:00",
+  "phone": "3331234567",
+  "email": "mario.rossi@example.com"
+}</t>
+  </si>
+  <si>
+    <t>Microsoft.Data.SqlClient.SqlException : Invalid column name 'DateOfBirth'.</t>
+  </si>
+  <si>
+    <t>TC07_CreatePatient_bug02.png</t>
+  </si>
+  <si>
+    <t>BUG02</t>
+  </si>
+  <si>
+    <t>TS2_20260321</t>
+  </si>
+  <si>
+    <t>{
+  "firstName": "Mario",
+  "lastName": "Rossi",
+  "taxCode": "RSSMRA85D12H501X",
+  "birthDate": "1985-04-12T00:00:00",
+  "phone": "3331234567",
+  "email": "mario.rossi@example.com"
+}</t>
+  </si>
+  <si>
+    <t>Paziente creato correttamente con ID:3</t>
+  </si>
+  <si>
+    <t>TC07_CreatePatient_Success.png</t>
   </si>
 </sst>
 </file>
@@ -1078,7 +1118,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1098,13 +1138,13 @@
     <xf numFmtId="0" fontId="13" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1113,8 +1153,11 @@
     <xf numFmtId="0" fontId="13" fillId="33" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1161,7 +1204,49 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="38">
+  <dxfs count="67">
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1177,6 +1262,48 @@
       </fill>
     </dxf>
     <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill>
           <bgColor rgb="FFFF0000"/>
@@ -1186,6 +1313,34 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
@@ -1212,40 +1367,19 @@
       </fill>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1330,42 +1464,84 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5E234CF2-B3FB-42E4-9C2F-2101E3219E96}" name="Table1" displayName="Table1" ref="A1:L24" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5E234CF2-B3FB-42E4-9C2F-2101E3219E96}" name="Table1" displayName="Table1" ref="A1:L24" totalsRowShown="0" headerRowDxfId="66" dataDxfId="65">
   <autoFilter ref="A1:L24" xr:uid="{5E234CF2-B3FB-42E4-9C2F-2101E3219E96}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{3860FCCE-8AB2-4BA5-A927-55A78AF301A2}" name="ID Test" dataDxfId="35"/>
-    <tableColumn id="2" xr3:uid="{6B8298D4-C558-435B-BC50-DF9FF417402B}" name="Area" dataDxfId="34"/>
-    <tableColumn id="3" xr3:uid="{53DE22B4-8437-4EA6-813E-2F0CF7E72133}" name="Obiettivo" dataDxfId="33"/>
-    <tableColumn id="4" xr3:uid="{59024008-94B6-47E6-8C7F-69725DFAE6EC}" name="Endpoint" dataDxfId="32"/>
-    <tableColumn id="5" xr3:uid="{DC8ACE73-D608-4E52-81FB-F85282B31F51}" name="Metodo HTTP" dataDxfId="31"/>
-    <tableColumn id="6" xr3:uid="{E583E0AB-6285-4FCA-BC35-0CD0BFB6F457}" name="Payload JSON" dataDxfId="30"/>
-    <tableColumn id="7" xr3:uid="{5BDBA1B2-61ED-47D6-88D1-CDE3D8CC9212}" name="Risultato atteso - Status Code" dataDxfId="29"/>
-    <tableColumn id="8" xr3:uid="{F14E32B9-432F-43ED-9E31-411BF4ADBC3F}" name="Risultato atteso - Dettaglio" dataDxfId="28"/>
-    <tableColumn id="9" xr3:uid="{DFDF46B3-7AFF-4643-9EAB-E56F926CE154}" name="Esito" dataDxfId="27"/>
-    <tableColumn id="10" xr3:uid="{5192CEE0-B98B-4E21-8BEA-8F62C2DAC458}" name="Risultato ottenuto" dataDxfId="26"/>
-    <tableColumn id="11" xr3:uid="{E9C64C9D-7B98-4D7D-8A82-64CB9D831A1C}" name="Screenshot" dataDxfId="25"/>
-    <tableColumn id="12" xr3:uid="{D98AF63F-322C-4828-B53E-197F74FEE6FE}" name="Note" dataDxfId="24"/>
+    <tableColumn id="1" xr3:uid="{3860FCCE-8AB2-4BA5-A927-55A78AF301A2}" name="ID Test" dataDxfId="64"/>
+    <tableColumn id="2" xr3:uid="{6B8298D4-C558-435B-BC50-DF9FF417402B}" name="Area" dataDxfId="63"/>
+    <tableColumn id="3" xr3:uid="{53DE22B4-8437-4EA6-813E-2F0CF7E72133}" name="Obiettivo" dataDxfId="62"/>
+    <tableColumn id="4" xr3:uid="{59024008-94B6-47E6-8C7F-69725DFAE6EC}" name="Endpoint" dataDxfId="61"/>
+    <tableColumn id="5" xr3:uid="{DC8ACE73-D608-4E52-81FB-F85282B31F51}" name="Metodo HTTP" dataDxfId="60"/>
+    <tableColumn id="6" xr3:uid="{E583E0AB-6285-4FCA-BC35-0CD0BFB6F457}" name="Payload JSON" dataDxfId="59"/>
+    <tableColumn id="7" xr3:uid="{5BDBA1B2-61ED-47D6-88D1-CDE3D8CC9212}" name="Risultato atteso - Status Code" dataDxfId="58"/>
+    <tableColumn id="8" xr3:uid="{F14E32B9-432F-43ED-9E31-411BF4ADBC3F}" name="Risultato atteso - Dettaglio" dataDxfId="57"/>
+    <tableColumn id="9" xr3:uid="{DFDF46B3-7AFF-4643-9EAB-E56F926CE154}" name="Esito" dataDxfId="56"/>
+    <tableColumn id="10" xr3:uid="{5192CEE0-B98B-4E21-8BEA-8F62C2DAC458}" name="Risultato ottenuto" dataDxfId="55"/>
+    <tableColumn id="11" xr3:uid="{E9C64C9D-7B98-4D7D-8A82-64CB9D831A1C}" name="Screenshot" dataDxfId="54"/>
+    <tableColumn id="12" xr3:uid="{D98AF63F-322C-4828-B53E-197F74FEE6FE}" name="Note" dataDxfId="53"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5EC5406F-ABEC-4C5A-BB6C-648C616B89A5}" name="Table13" displayName="Table13" ref="A1:L24" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5EC5406F-ABEC-4C5A-BB6C-648C616B89A5}" name="Table13" displayName="Table13" ref="A1:L24" totalsRowShown="0" headerRowDxfId="52" dataDxfId="51">
   <autoFilter ref="A1:L24" xr:uid="{5E234CF2-B3FB-42E4-9C2F-2101E3219E96}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{5009D189-63E8-4852-A288-87D6EC1E7033}" name="ID Test" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{84642470-32B1-46DB-88F2-1BC4AE8F75C8}" name="Area" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{4F14914F-A3C4-4267-A392-EC2D02D6ADDF}" name="Obiettivo" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{62A87606-C1B8-47E6-9530-D288374DCDF3}" name="Endpoint" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{19E09EE6-EB67-45CF-9A03-E0F0523DB6A0}" name="Metodo HTTP" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{A7AC84FA-A2F1-4930-BDDD-E380EE204368}" name="Payload JSON" dataDxfId="16"/>
-    <tableColumn id="7" xr3:uid="{25C18B10-E594-4E87-AD84-2A557086D8F7}" name="Risultato atteso - Status Code" dataDxfId="15"/>
-    <tableColumn id="8" xr3:uid="{94B79096-6200-43FE-8F50-1C48EB575740}" name="Risultato atteso - Dettaglio" dataDxfId="12"/>
-    <tableColumn id="9" xr3:uid="{AD4E1447-793D-4E65-9313-6A19D961F6AE}" name="Esito" dataDxfId="10"/>
-    <tableColumn id="10" xr3:uid="{B18252F9-BB1D-47B7-8E2C-F42387EC3664}" name="Risultato ottenuto" dataDxfId="11"/>
-    <tableColumn id="11" xr3:uid="{15A8AB07-0563-4A1C-839B-92039F98E2D5}" name="Screenshot" dataDxfId="14"/>
-    <tableColumn id="12" xr3:uid="{4BA21C77-65A7-407A-A5E1-0AA6154386E8}" name="Note" dataDxfId="13"/>
+    <tableColumn id="1" xr3:uid="{5009D189-63E8-4852-A288-87D6EC1E7033}" name="ID Test" dataDxfId="50"/>
+    <tableColumn id="2" xr3:uid="{84642470-32B1-46DB-88F2-1BC4AE8F75C8}" name="Area" dataDxfId="49"/>
+    <tableColumn id="3" xr3:uid="{4F14914F-A3C4-4267-A392-EC2D02D6ADDF}" name="Obiettivo" dataDxfId="48"/>
+    <tableColumn id="4" xr3:uid="{62A87606-C1B8-47E6-9530-D288374DCDF3}" name="Endpoint" dataDxfId="47"/>
+    <tableColumn id="5" xr3:uid="{19E09EE6-EB67-45CF-9A03-E0F0523DB6A0}" name="Metodo HTTP" dataDxfId="46"/>
+    <tableColumn id="6" xr3:uid="{A7AC84FA-A2F1-4930-BDDD-E380EE204368}" name="Payload JSON" dataDxfId="45"/>
+    <tableColumn id="7" xr3:uid="{25C18B10-E594-4E87-AD84-2A557086D8F7}" name="Risultato atteso - Status Code" dataDxfId="44"/>
+    <tableColumn id="8" xr3:uid="{94B79096-6200-43FE-8F50-1C48EB575740}" name="Risultato atteso - Dettaglio" dataDxfId="43"/>
+    <tableColumn id="9" xr3:uid="{AD4E1447-793D-4E65-9313-6A19D961F6AE}" name="Esito" dataDxfId="42"/>
+    <tableColumn id="10" xr3:uid="{B18252F9-BB1D-47B7-8E2C-F42387EC3664}" name="Risultato ottenuto" dataDxfId="41"/>
+    <tableColumn id="11" xr3:uid="{15A8AB07-0563-4A1C-839B-92039F98E2D5}" name="Screenshot" dataDxfId="40"/>
+    <tableColumn id="12" xr3:uid="{4BA21C77-65A7-407A-A5E1-0AA6154386E8}" name="Note" dataDxfId="39"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{3C84183B-2219-4217-B03E-3888C2A1762E}" name="Table134" displayName="Table134" ref="A1:L24" totalsRowShown="0" headerRowDxfId="29" dataDxfId="28">
+  <autoFilter ref="A1:L24" xr:uid="{5E234CF2-B3FB-42E4-9C2F-2101E3219E96}"/>
+  <tableColumns count="12">
+    <tableColumn id="1" xr3:uid="{B704E338-5C37-41FB-8C85-99D253E12A36}" name="ID Test" dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{B2981A3F-A838-4564-95CD-018029141FE3}" name="Area" dataDxfId="26"/>
+    <tableColumn id="3" xr3:uid="{3A09ED62-C911-40F8-84B2-95FDC9F0E73C}" name="Obiettivo" dataDxfId="25"/>
+    <tableColumn id="4" xr3:uid="{7D97DC0F-3E73-4208-8A63-D6DE3FC761AA}" name="Endpoint" dataDxfId="24"/>
+    <tableColumn id="5" xr3:uid="{FF0C5D75-36E7-48D4-A80F-888A5CC255B7}" name="Metodo HTTP" dataDxfId="23"/>
+    <tableColumn id="6" xr3:uid="{023149CE-2E87-48C5-89F0-C06C9BB739DA}" name="Payload JSON" dataDxfId="22"/>
+    <tableColumn id="7" xr3:uid="{8BAEE933-7939-4263-9D14-00FEC91A9C1B}" name="Risultato atteso - Status Code" dataDxfId="21"/>
+    <tableColumn id="8" xr3:uid="{8D31C62B-63D8-4839-9FA3-50CF6221E2BA}" name="Risultato atteso - Dettaglio" dataDxfId="20"/>
+    <tableColumn id="9" xr3:uid="{718B97BF-78C2-4F95-B210-9079004CD606}" name="Esito" dataDxfId="19"/>
+    <tableColumn id="10" xr3:uid="{5CFD81E3-BB64-412E-85AA-84B4611A7F83}" name="Risultato ottenuto" dataDxfId="18"/>
+    <tableColumn id="11" xr3:uid="{6A9BDE4A-CBAC-4363-A060-8EA060236295}" name="Screenshot" dataDxfId="17"/>
+    <tableColumn id="12" xr3:uid="{4E358191-7A4E-4452-AC66-1FBA8A472BD5}" name="Note" dataDxfId="16"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{5392533B-6B0E-4F8C-A890-54E0F381453F}" name="Table1345" displayName="Table1345" ref="A1:L24" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+  <autoFilter ref="A1:L24" xr:uid="{5E234CF2-B3FB-42E4-9C2F-2101E3219E96}"/>
+  <tableColumns count="12">
+    <tableColumn id="1" xr3:uid="{5DB9B359-E545-4837-92D9-C3F683AC6170}" name="ID Test" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{3357AA3D-D573-45C9-9E54-169DE6BCCC7B}" name="Area" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{FE4BC87A-DD7A-4AC5-9DF0-39C04CF1DEDC}" name="Obiettivo" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{61F99A4D-AC1D-4AAE-BD37-39FC313ECF7E}" name="Endpoint" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{5FD12983-51FF-4BBD-B2DE-46FBD352051D}" name="Metodo HTTP" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{B67C064B-9915-4F2D-8311-0F58E542AA8C}" name="Payload JSON" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{8875AB99-AAA8-46E7-8416-18C1D1E6E0D6}" name="Risultato atteso - Status Code" dataDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{6DA0A166-C4F1-4D89-874B-4007FF063015}" name="Risultato atteso - Dettaglio" dataDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{C4E9099C-524E-4645-AE6E-B8ACEAF227A2}" name="Esito" dataDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{8329D30F-DF3B-4467-8F69-F9BE9E265DCA}" name="Risultato ottenuto" dataDxfId="2"/>
+    <tableColumn id="11" xr3:uid="{99A837AC-AC32-4D7E-BCA2-CEC29E347BE5}" name="Screenshot" dataDxfId="1"/>
+    <tableColumn id="12" xr3:uid="{05FA14BC-760C-4AFA-975E-E185779DFF89}" name="Note" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2354,10 +2530,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="I2:I24">
-    <cfRule type="cellIs" dxfId="6" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="38" priority="1" operator="equal">
       <formula>"OK"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="37" priority="2" operator="equal">
       <formula>"KO"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2376,7 +2552,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27CCBE7D-F26A-41C6-96A8-43D2BF97BCE3}">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultColWidth="91.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.7109375" bestFit="1" customWidth="1"/>
@@ -2454,20 +2630,50 @@
         <v>135</v>
       </c>
     </row>
+    <row r="3" spans="1:10" ht="120" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>162</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="H3" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="I3" s="13" t="s">
+        <v>166</v>
+      </c>
+      <c r="J3" s="13" t="s">
+        <v>167</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="D2">
-    <cfRule type="cellIs" dxfId="4" priority="1" operator="equal">
+  <conditionalFormatting sqref="D2:D3">
+    <cfRule type="cellIs" dxfId="36" priority="1" operator="equal">
       <formula>"BASSA"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="35" priority="2" operator="equal">
       <formula>"MEDIA"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="34" priority="3" operator="equal">
       <formula>"ALTA"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2" xr:uid="{78C482C4-A569-4755-A44B-F5FA399B9D9D}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D3" xr:uid="{78C482C4-A569-4755-A44B-F5FA399B9D9D}">
       <formula1>"ALTA,MEDIA,BASSA"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3262,10 +3468,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="I2:I24">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="33" priority="1" operator="equal">
       <formula>"OK"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="32" priority="2" operator="equal">
       <formula>"KO"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3280,4 +3486,1615 @@
     <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C20C51C6-6E6F-4215-9FA0-CAF40473805B}">
+  <dimension ref="A1:L24"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="15.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="85.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="36.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="54.7109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="29" style="2" customWidth="1"/>
+    <col min="8" max="8" width="41.7109375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="7.42578125" style="4" customWidth="1"/>
+    <col min="10" max="10" width="41.7109375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="58.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="64" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="9.140625" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="120" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="L13" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="L15" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="I20" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="J20" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="K20" s="2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="J21" s="1" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="L22" s="1" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="L23" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="K24" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="L24" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="I2:I24">
+    <cfRule type="cellIs" dxfId="31" priority="1" operator="equal">
+      <formula>"OK"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="30" priority="2" operator="equal">
+      <formula>"KO"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I24" xr:uid="{D757978B-CD58-47E6-82A0-86878BFDB70A}">
+      <formula1>"OK,KO"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2BEB9BE-D1E1-427B-A8AB-8E7466BA14C6}">
+  <dimension ref="A1:L24"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="15.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="85.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="36.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="54.7109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="29" style="2" customWidth="1"/>
+    <col min="8" max="8" width="41.7109375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="7.42578125" style="4" customWidth="1"/>
+    <col min="10" max="10" width="41.7109375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="58.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="64" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="9.140625" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="120" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="L13" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="L15" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="I20" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="J20" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="K20" s="2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="J21" s="1" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="L22" s="1" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="L23" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="K24" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="L24" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="I2:I24">
+    <cfRule type="cellIs" dxfId="15" priority="1" operator="equal">
+      <formula>"OK"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="14" priority="2" operator="equal">
+      <formula>"KO"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I24" xr:uid="{C6C44458-0CCE-4CF1-A06A-1FBD3698EB51}">
+      <formula1>"OK,KO"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Registrato esito ok dei bug in testbook
</commit_message>
<xml_diff>
--- a/docs/testbook/ClinicaFlow_TestBook_API.xlsx
+++ b/docs/testbook/ClinicaFlow_TestBook_API.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\valen\clinicaflow\docs\testbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99819984-289C-4DA6-AE98-9D390E4B0077}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83976FBE-77E6-4384-9BBB-69792E27FE2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20370" yWindow="-4770" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{1C9960E8-B103-4EFA-9509-2FD0D5F86CF0}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="950" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="952" uniqueCount="175">
   <si>
     <t>ID Test</t>
   </si>
@@ -560,6 +560,9 @@
   </si>
   <si>
     <t>TC07_CreatePatient_Success.png</t>
+  </si>
+  <si>
+    <t>TS3_20260321</t>
   </si>
 </sst>
 </file>
@@ -1118,7 +1121,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1155,9 +1158,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1206,48 +1206,6 @@
   </cellStyles>
   <dxfs count="67">
     <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill>
           <bgColor rgb="FFFF0000"/>
@@ -1262,48 +1220,6 @@
       </fill>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill>
           <bgColor rgb="FFFF0000"/>
@@ -1365,6 +1281,90 @@
           <bgColor rgb="FF92D050"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1506,42 +1506,42 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{3C84183B-2219-4217-B03E-3888C2A1762E}" name="Table134" displayName="Table134" ref="A1:L24" totalsRowShown="0" headerRowDxfId="29" dataDxfId="28">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{3C84183B-2219-4217-B03E-3888C2A1762E}" name="Table134" displayName="Table134" ref="A1:L24" totalsRowShown="0" headerRowDxfId="38" dataDxfId="37">
   <autoFilter ref="A1:L24" xr:uid="{5E234CF2-B3FB-42E4-9C2F-2101E3219E96}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{B704E338-5C37-41FB-8C85-99D253E12A36}" name="ID Test" dataDxfId="27"/>
-    <tableColumn id="2" xr3:uid="{B2981A3F-A838-4564-95CD-018029141FE3}" name="Area" dataDxfId="26"/>
-    <tableColumn id="3" xr3:uid="{3A09ED62-C911-40F8-84B2-95FDC9F0E73C}" name="Obiettivo" dataDxfId="25"/>
-    <tableColumn id="4" xr3:uid="{7D97DC0F-3E73-4208-8A63-D6DE3FC761AA}" name="Endpoint" dataDxfId="24"/>
-    <tableColumn id="5" xr3:uid="{FF0C5D75-36E7-48D4-A80F-888A5CC255B7}" name="Metodo HTTP" dataDxfId="23"/>
-    <tableColumn id="6" xr3:uid="{023149CE-2E87-48C5-89F0-C06C9BB739DA}" name="Payload JSON" dataDxfId="22"/>
-    <tableColumn id="7" xr3:uid="{8BAEE933-7939-4263-9D14-00FEC91A9C1B}" name="Risultato atteso - Status Code" dataDxfId="21"/>
-    <tableColumn id="8" xr3:uid="{8D31C62B-63D8-4839-9FA3-50CF6221E2BA}" name="Risultato atteso - Dettaglio" dataDxfId="20"/>
-    <tableColumn id="9" xr3:uid="{718B97BF-78C2-4F95-B210-9079004CD606}" name="Esito" dataDxfId="19"/>
-    <tableColumn id="10" xr3:uid="{5CFD81E3-BB64-412E-85AA-84B4611A7F83}" name="Risultato ottenuto" dataDxfId="18"/>
-    <tableColumn id="11" xr3:uid="{6A9BDE4A-CBAC-4363-A060-8EA060236295}" name="Screenshot" dataDxfId="17"/>
-    <tableColumn id="12" xr3:uid="{4E358191-7A4E-4452-AC66-1FBA8A472BD5}" name="Note" dataDxfId="16"/>
+    <tableColumn id="1" xr3:uid="{B704E338-5C37-41FB-8C85-99D253E12A36}" name="ID Test" dataDxfId="36"/>
+    <tableColumn id="2" xr3:uid="{B2981A3F-A838-4564-95CD-018029141FE3}" name="Area" dataDxfId="35"/>
+    <tableColumn id="3" xr3:uid="{3A09ED62-C911-40F8-84B2-95FDC9F0E73C}" name="Obiettivo" dataDxfId="34"/>
+    <tableColumn id="4" xr3:uid="{7D97DC0F-3E73-4208-8A63-D6DE3FC761AA}" name="Endpoint" dataDxfId="33"/>
+    <tableColumn id="5" xr3:uid="{FF0C5D75-36E7-48D4-A80F-888A5CC255B7}" name="Metodo HTTP" dataDxfId="32"/>
+    <tableColumn id="6" xr3:uid="{023149CE-2E87-48C5-89F0-C06C9BB739DA}" name="Payload JSON" dataDxfId="31"/>
+    <tableColumn id="7" xr3:uid="{8BAEE933-7939-4263-9D14-00FEC91A9C1B}" name="Risultato atteso - Status Code" dataDxfId="30"/>
+    <tableColumn id="8" xr3:uid="{8D31C62B-63D8-4839-9FA3-50CF6221E2BA}" name="Risultato atteso - Dettaglio" dataDxfId="29"/>
+    <tableColumn id="9" xr3:uid="{718B97BF-78C2-4F95-B210-9079004CD606}" name="Esito" dataDxfId="28"/>
+    <tableColumn id="10" xr3:uid="{5CFD81E3-BB64-412E-85AA-84B4611A7F83}" name="Risultato ottenuto" dataDxfId="27"/>
+    <tableColumn id="11" xr3:uid="{6A9BDE4A-CBAC-4363-A060-8EA060236295}" name="Screenshot" dataDxfId="26"/>
+    <tableColumn id="12" xr3:uid="{4E358191-7A4E-4452-AC66-1FBA8A472BD5}" name="Note" dataDxfId="25"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{5392533B-6B0E-4F8C-A890-54E0F381453F}" name="Table1345" displayName="Table1345" ref="A1:L24" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{5392533B-6B0E-4F8C-A890-54E0F381453F}" name="Table1345" displayName="Table1345" ref="A1:L24" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
   <autoFilter ref="A1:L24" xr:uid="{5E234CF2-B3FB-42E4-9C2F-2101E3219E96}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{5DB9B359-E545-4837-92D9-C3F683AC6170}" name="ID Test" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{3357AA3D-D573-45C9-9E54-169DE6BCCC7B}" name="Area" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{FE4BC87A-DD7A-4AC5-9DF0-39C04CF1DEDC}" name="Obiettivo" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{61F99A4D-AC1D-4AAE-BD37-39FC313ECF7E}" name="Endpoint" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{5FD12983-51FF-4BBD-B2DE-46FBD352051D}" name="Metodo HTTP" dataDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{B67C064B-9915-4F2D-8311-0F58E542AA8C}" name="Payload JSON" dataDxfId="6"/>
-    <tableColumn id="7" xr3:uid="{8875AB99-AAA8-46E7-8416-18C1D1E6E0D6}" name="Risultato atteso - Status Code" dataDxfId="5"/>
-    <tableColumn id="8" xr3:uid="{6DA0A166-C4F1-4D89-874B-4007FF063015}" name="Risultato atteso - Dettaglio" dataDxfId="4"/>
-    <tableColumn id="9" xr3:uid="{C4E9099C-524E-4645-AE6E-B8ACEAF227A2}" name="Esito" dataDxfId="3"/>
-    <tableColumn id="10" xr3:uid="{8329D30F-DF3B-4467-8F69-F9BE9E265DCA}" name="Risultato ottenuto" dataDxfId="2"/>
-    <tableColumn id="11" xr3:uid="{99A837AC-AC32-4D7E-BCA2-CEC29E347BE5}" name="Screenshot" dataDxfId="1"/>
-    <tableColumn id="12" xr3:uid="{05FA14BC-760C-4AFA-975E-E185779DFF89}" name="Note" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{5DB9B359-E545-4837-92D9-C3F683AC6170}" name="ID Test" dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{3357AA3D-D573-45C9-9E54-169DE6BCCC7B}" name="Area" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{FE4BC87A-DD7A-4AC5-9DF0-39C04CF1DEDC}" name="Obiettivo" dataDxfId="20"/>
+    <tableColumn id="4" xr3:uid="{61F99A4D-AC1D-4AAE-BD37-39FC313ECF7E}" name="Endpoint" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{5FD12983-51FF-4BBD-B2DE-46FBD352051D}" name="Metodo HTTP" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{B67C064B-9915-4F2D-8311-0F58E542AA8C}" name="Payload JSON" dataDxfId="17"/>
+    <tableColumn id="7" xr3:uid="{8875AB99-AAA8-46E7-8416-18C1D1E6E0D6}" name="Risultato atteso - Status Code" dataDxfId="16"/>
+    <tableColumn id="8" xr3:uid="{6DA0A166-C4F1-4D89-874B-4007FF063015}" name="Risultato atteso - Dettaglio" dataDxfId="15"/>
+    <tableColumn id="9" xr3:uid="{C4E9099C-524E-4645-AE6E-B8ACEAF227A2}" name="Esito" dataDxfId="14"/>
+    <tableColumn id="10" xr3:uid="{8329D30F-DF3B-4467-8F69-F9BE9E265DCA}" name="Risultato ottenuto" dataDxfId="13"/>
+    <tableColumn id="11" xr3:uid="{99A837AC-AC32-4D7E-BCA2-CEC29E347BE5}" name="Screenshot" dataDxfId="12"/>
+    <tableColumn id="12" xr3:uid="{05FA14BC-760C-4AFA-975E-E185779DFF89}" name="Note" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2530,10 +2530,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="I2:I24">
-    <cfRule type="cellIs" dxfId="38" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="1" operator="equal">
       <formula>"OK"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="2" operator="equal">
       <formula>"KO"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2616,7 +2616,9 @@
       <c r="E2" s="8" t="s">
         <v>163</v>
       </c>
-      <c r="F2" s="8"/>
+      <c r="F2" s="8" t="s">
+        <v>170</v>
+      </c>
       <c r="G2" s="8" t="s">
         <v>112</v>
       </c>
@@ -2646,29 +2648,31 @@
       <c r="E3" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="F3" s="8"/>
+      <c r="F3" s="8" t="s">
+        <v>174</v>
+      </c>
       <c r="G3" s="8" t="s">
         <v>112</v>
       </c>
       <c r="H3" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="13" t="s">
+      <c r="I3" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="J3" s="13" t="s">
+      <c r="J3" s="9" t="s">
         <v>167</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="D2:D3">
-    <cfRule type="cellIs" dxfId="36" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
       <formula>"BASSA"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="35" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="2" operator="equal">
       <formula>"MEDIA"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="34" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="3" operator="equal">
       <formula>"ALTA"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3468,10 +3472,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="I2:I24">
-    <cfRule type="cellIs" dxfId="33" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
       <formula>"OK"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="32" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
       <formula>"KO"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4275,10 +4279,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="I2:I24">
-    <cfRule type="cellIs" dxfId="31" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>"OK"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
       <formula>"KO"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5079,10 +5083,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="I2:I24">
-    <cfRule type="cellIs" dxfId="15" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"OK"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
       <formula>"KO"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>